<commit_message>
Add pii column to survey editing template
</commit_message>
<xml_diff>
--- a/fieldManagerClient/WebContent/blankform.xlsx
+++ b/fieldManagerClient/WebContent/blankform.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10517"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neilpenman/git/prop-smapserver/fieldManagerClient/WebContent/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{555B6DA2-2CB2-E047-9B8E-864FB036E234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96F55A40-4F6E-1E45-BC5B-99A00C7028DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="920" windowWidth="30680" windowHeight="13220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="115">
   <si>
     <t>type</t>
   </si>
@@ -383,6 +383,9 @@
   </si>
   <si>
     <t>Calculations that are done on the server when the data is viewed</t>
+  </si>
+  <si>
+    <t>pii</t>
   </si>
 </sst>
 </file>
@@ -813,15 +816,15 @@
   <sheetPr>
     <tabColor theme="6" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="26" width="20" customWidth="1"/>
+    <col min="4" max="27" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -871,33 +874,36 @@
         <v>12</v>
       </c>
       <c r="Q1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1567,4 +1573,10 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{11067652-e594-4683-81e3-2cbf4d08314b}" enabled="1" method="Standard" siteId="{dd4b51f9-ee38-4f0d-87d3-0fcc190484cf}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>